<commit_message>
Update Reliability Project 1 Files
</commit_message>
<xml_diff>
--- a/Reliability/project1/data/课题一/Stochastic_Process_Models_Evaluation.xlsx
+++ b/Reliability/project1/data/课题一/Stochastic_Process_Models_Evaluation.xlsx
@@ -472,13 +472,13 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>69.63517940944723</v>
+        <v>69.63517940934219</v>
       </c>
       <c r="D3" t="n">
-        <v>-135.2703588188945</v>
+        <v>-135.2703588186844</v>
       </c>
       <c r="E3" t="n">
-        <v>-128.3090809722105</v>
+        <v>-128.3090809720004</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>75.11540943195459</v>
+        <v>75.11540892370074</v>
       </c>
       <c r="D4" t="n">
-        <v>-146.2308188639092</v>
+        <v>-146.2308178474015</v>
       </c>
       <c r="E4" t="n">
-        <v>-139.2695410172252</v>
+        <v>-139.2695400007175</v>
       </c>
     </row>
     <row r="5">

</xml_diff>